<commit_message>
Fix NS-0755 mapping in withdrawals review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA2XXv3viuKc4AVC546mfn
</commit_message>
<xml_diff>
--- a/مراجعة_شيتات_المسحوبات_الرياض_تبوك.xlsx
+++ b/مراجعة_شيتات_المسحوبات_الرياض_تبوك.xlsx
@@ -19,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy/mm/dd"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -102,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -125,17 +124,23 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -625,7 +630,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D9" s="3" t="inlineStr"/>
     </row>
@@ -653,7 +658,7 @@
         <v>8</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D11" s="3" t="inlineStr"/>
     </row>
@@ -844,7 +849,7 @@
       <c r="A2" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B2" s="10" t="n">
+      <c r="B2" s="21" t="n">
         <v>46239</v>
       </c>
       <c r="C2" s="9" t="inlineStr">
@@ -890,7 +895,7 @@
       <c r="A3" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B3" s="10" t="n">
+      <c r="B3" s="21" t="n">
         <v>46239</v>
       </c>
       <c r="C3" s="9" t="inlineStr">
@@ -930,7 +935,7 @@
       <c r="A4" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="21" t="n">
         <v>46239</v>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -970,7 +975,7 @@
       <c r="A5" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="21" t="n">
         <v>46239</v>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -1010,7 +1015,7 @@
       <c r="A6" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="21" t="n">
         <v>46239</v>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -1050,7 +1055,7 @@
       <c r="A7" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="21" t="n">
         <v>46239</v>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -1090,7 +1095,7 @@
       <c r="A8" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="21" t="n">
         <v>45969</v>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -1132,7 +1137,7 @@
       <c r="A9" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="21" t="n">
         <v>45969</v>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -1172,7 +1177,7 @@
       <c r="A10" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="21" t="n">
         <v>45969</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -1212,7 +1217,7 @@
       <c r="A11" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="21" t="n">
         <v>45969</v>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -1252,7 +1257,7 @@
       <c r="A12" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="21" t="n">
         <v>45969</v>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -1292,7 +1297,7 @@
       <c r="A13" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="B13" s="10" t="n">
+      <c r="B13" s="21" t="n">
         <v>45981</v>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -1334,7 +1339,7 @@
       <c r="A14" s="9" t="n">
         <v>17</v>
       </c>
-      <c r="B14" s="10" t="n">
+      <c r="B14" s="21" t="n">
         <v>45981</v>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -1374,7 +1379,7 @@
       <c r="A15" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="21" t="n">
         <v>46002</v>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -1416,7 +1421,7 @@
       <c r="A16" s="9" t="n">
         <v>19</v>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="21" t="n">
         <v>46025</v>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -1462,7 +1467,7 @@
       <c r="A17" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="21" t="n">
         <v>46025</v>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -1502,7 +1507,7 @@
       <c r="A18" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B18" s="10" t="n">
+      <c r="B18" s="21" t="n">
         <v>46025</v>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -1542,7 +1547,7 @@
       <c r="A19" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B19" s="10" t="n">
+      <c r="B19" s="21" t="n">
         <v>46025</v>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -1582,7 +1587,7 @@
       <c r="A20" s="12" t="n">
         <v>23</v>
       </c>
-      <c r="B20" s="13" t="n">
+      <c r="B20" s="22" t="n">
         <v>46117</v>
       </c>
       <c r="C20" s="12" t="inlineStr">
@@ -1628,7 +1633,7 @@
       <c r="A21" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="B21" s="13" t="n"/>
+      <c r="B21" s="22" t="n"/>
       <c r="C21" s="12" t="inlineStr">
         <is>
           <t>فرق PO الشجيرات</t>
@@ -1672,7 +1677,7 @@
       <c r="A22" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="B22" s="13" t="n"/>
+      <c r="B22" s="22" t="n"/>
       <c r="C22" s="12" t="inlineStr">
         <is>
           <t>فرق PO الشجيرات</t>
@@ -1710,7 +1715,7 @@
       <c r="A23" s="12" t="n">
         <v>26</v>
       </c>
-      <c r="B23" s="13" t="n"/>
+      <c r="B23" s="22" t="n"/>
       <c r="C23" s="12" t="inlineStr">
         <is>
           <t>فرق PO الشجيرات</t>
@@ -1748,7 +1753,7 @@
       <c r="A24" s="12" t="n">
         <v>27</v>
       </c>
-      <c r="B24" s="13" t="n"/>
+      <c r="B24" s="22" t="n"/>
       <c r="C24" s="12" t="inlineStr">
         <is>
           <t>فرق PO الشجيرات</t>
@@ -1786,7 +1791,7 @@
       <c r="A25" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="B25" s="13" t="n"/>
+      <c r="B25" s="22" t="n"/>
       <c r="C25" s="12" t="inlineStr">
         <is>
           <t>فرق PO الشجيرات</t>
@@ -1824,7 +1829,7 @@
       <c r="A26" s="12" t="n">
         <v>29</v>
       </c>
-      <c r="B26" s="13" t="n"/>
+      <c r="B26" s="22" t="n"/>
       <c r="C26" s="12" t="inlineStr">
         <is>
           <t>فرق PO الشجيرات</t>
@@ -1862,7 +1867,7 @@
       <c r="A27" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="B27" s="13" t="n"/>
+      <c r="B27" s="22" t="n"/>
       <c r="C27" s="12" t="inlineStr">
         <is>
           <t>فرق PO الشجيرات</t>
@@ -2004,7 +2009,7 @@
       <c r="A2" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B2" s="10" t="n">
+      <c r="B2" s="21" t="n">
         <v>45906</v>
       </c>
       <c r="C2" s="9" t="inlineStr">
@@ -2046,7 +2051,7 @@
       <c r="A3" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B3" s="10" t="n">
+      <c r="B3" s="21" t="n">
         <v>45926</v>
       </c>
       <c r="C3" s="9" t="inlineStr">
@@ -2088,7 +2093,7 @@
       <c r="A4" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="21" t="n">
         <v>45926</v>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -2128,7 +2133,7 @@
       <c r="A5" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="21" t="n">
         <v>45926</v>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -2168,7 +2173,7 @@
       <c r="A6" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="21" t="n">
         <v>45926</v>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -2210,7 +2215,7 @@
       <c r="A7" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="21" t="n">
         <v>45937</v>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -2256,7 +2261,7 @@
       <c r="A8" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="21" t="n">
         <v>45937</v>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -2296,7 +2301,7 @@
       <c r="A9" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="21" t="n">
         <v>45937</v>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -2336,7 +2341,7 @@
       <c r="A10" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="21" t="n">
         <v>45937</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -2376,7 +2381,7 @@
       <c r="A11" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="21" t="n">
         <v>45937</v>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -2416,7 +2421,7 @@
       <c r="A12" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="21" t="n">
         <v>45937</v>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -2456,7 +2461,7 @@
       <c r="A13" s="9" t="n">
         <v>17</v>
       </c>
-      <c r="B13" s="10" t="n">
+      <c r="B13" s="21" t="n">
         <v>45937</v>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -2496,7 +2501,7 @@
       <c r="A14" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="B14" s="10" t="n">
+      <c r="B14" s="21" t="n">
         <v>45937</v>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -2536,7 +2541,7 @@
       <c r="A15" s="9" t="n">
         <v>19</v>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="21" t="n">
         <v>45947</v>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -2578,7 +2583,7 @@
       <c r="A16" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="21" t="n">
         <v>45947</v>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -2618,7 +2623,7 @@
       <c r="A17" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="21" t="n">
         <v>45947</v>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -2658,7 +2663,7 @@
       <c r="A18" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B18" s="10" t="n">
+      <c r="B18" s="21" t="n">
         <v>45954</v>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -2700,7 +2705,7 @@
       <c r="A19" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="B19" s="10" t="n">
+      <c r="B19" s="21" t="n">
         <v>45962</v>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -2742,7 +2747,7 @@
       <c r="A20" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="21" t="n">
         <v>45962</v>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -2782,7 +2787,7 @@
       <c r="A21" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="21" t="n">
         <v>45962</v>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -2822,7 +2827,7 @@
       <c r="A22" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B22" s="10" t="n">
+      <c r="B22" s="21" t="n">
         <v>45962</v>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -2862,7 +2867,7 @@
       <c r="A23" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="B23" s="10" t="n">
+      <c r="B23" s="21" t="n">
         <v>45964</v>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -2904,7 +2909,7 @@
       <c r="A24" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="B24" s="10" t="n">
+      <c r="B24" s="21" t="n">
         <v>45969</v>
       </c>
       <c r="C24" s="9" t="inlineStr">
@@ -2946,7 +2951,7 @@
       <c r="A25" s="9" t="n">
         <v>29</v>
       </c>
-      <c r="B25" s="10" t="n">
+      <c r="B25" s="21" t="n">
         <v>45969</v>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -2986,7 +2991,7 @@
       <c r="A26" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B26" s="10" t="n">
+      <c r="B26" s="21" t="n">
         <v>45999</v>
       </c>
       <c r="C26" s="9" t="inlineStr">
@@ -3028,7 +3033,7 @@
       <c r="A27" s="9" t="n">
         <v>31</v>
       </c>
-      <c r="B27" s="10" t="n">
+      <c r="B27" s="21" t="n">
         <v>45999</v>
       </c>
       <c r="C27" s="9" t="inlineStr">
@@ -3070,7 +3075,7 @@
       <c r="A28" s="9" t="n">
         <v>32</v>
       </c>
-      <c r="B28" s="10" t="n">
+      <c r="B28" s="21" t="n">
         <v>46011</v>
       </c>
       <c r="C28" s="9" t="inlineStr">
@@ -3112,7 +3117,7 @@
       <c r="A29" s="9" t="n">
         <v>33</v>
       </c>
-      <c r="B29" s="10" t="n">
+      <c r="B29" s="21" t="n">
         <v>46011</v>
       </c>
       <c r="C29" s="9" t="inlineStr">
@@ -3152,7 +3157,7 @@
       <c r="A30" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="B30" s="10" t="n">
+      <c r="B30" s="21" t="n">
         <v>46011</v>
       </c>
       <c r="C30" s="9" t="inlineStr">
@@ -3192,7 +3197,7 @@
       <c r="A31" s="17" t="n">
         <v>35</v>
       </c>
-      <c r="B31" s="18" t="n">
+      <c r="B31" s="23" t="n">
         <v>46026</v>
       </c>
       <c r="C31" s="17" t="inlineStr">
@@ -3234,7 +3239,7 @@
       <c r="A32" s="17" t="n">
         <v>36</v>
       </c>
-      <c r="B32" s="18" t="n">
+      <c r="B32" s="23" t="n">
         <v>46026</v>
       </c>
       <c r="C32" s="17" t="inlineStr">
@@ -3274,7 +3279,7 @@
       <c r="A33" s="17" t="n">
         <v>37</v>
       </c>
-      <c r="B33" s="18" t="n">
+      <c r="B33" s="23" t="n">
         <v>46026</v>
       </c>
       <c r="C33" s="17" t="inlineStr">
@@ -3316,7 +3321,7 @@
       <c r="A34" s="17" t="n">
         <v>38</v>
       </c>
-      <c r="B34" s="18" t="n">
+      <c r="B34" s="23" t="n">
         <v>46026</v>
       </c>
       <c r="C34" s="17" t="inlineStr">
@@ -3356,7 +3361,7 @@
       <c r="A35" s="17" t="n">
         <v>39</v>
       </c>
-      <c r="B35" s="18" t="n">
+      <c r="B35" s="23" t="n">
         <v>46026</v>
       </c>
       <c r="C35" s="17" t="inlineStr">
@@ -3396,7 +3401,7 @@
       <c r="A36" s="17" t="n">
         <v>40</v>
       </c>
-      <c r="B36" s="18" t="n">
+      <c r="B36" s="23" t="n">
         <v>46026</v>
       </c>
       <c r="C36" s="17" t="inlineStr">
@@ -3436,7 +3441,7 @@
       <c r="A37" s="17" t="n">
         <v>41</v>
       </c>
-      <c r="B37" s="18" t="n">
+      <c r="B37" s="23" t="n">
         <v>46026</v>
       </c>
       <c r="C37" s="17" t="inlineStr">
@@ -3478,7 +3483,7 @@
       <c r="A38" s="17" t="n">
         <v>42</v>
       </c>
-      <c r="B38" s="18" t="n">
+      <c r="B38" s="23" t="n">
         <v>46029</v>
       </c>
       <c r="C38" s="17" t="inlineStr">
@@ -3520,7 +3525,7 @@
       <c r="A39" s="17" t="n">
         <v>43</v>
       </c>
-      <c r="B39" s="18" t="n">
+      <c r="B39" s="23" t="n">
         <v>46029</v>
       </c>
       <c r="C39" s="17" t="inlineStr">
@@ -3560,7 +3565,7 @@
       <c r="A40" s="17" t="n">
         <v>44</v>
       </c>
-      <c r="B40" s="18" t="n">
+      <c r="B40" s="23" t="n">
         <v>46029</v>
       </c>
       <c r="C40" s="17" t="inlineStr">
@@ -3600,7 +3605,7 @@
       <c r="A41" s="17" t="n">
         <v>45</v>
       </c>
-      <c r="B41" s="18" t="n">
+      <c r="B41" s="23" t="n">
         <v>46033</v>
       </c>
       <c r="C41" s="17" t="inlineStr">
@@ -3642,7 +3647,7 @@
       <c r="A42" s="9" t="n">
         <v>46</v>
       </c>
-      <c r="B42" s="10" t="n">
+      <c r="B42" s="21" t="n">
         <v>46040</v>
       </c>
       <c r="C42" s="9" t="inlineStr">
@@ -3684,7 +3689,7 @@
       <c r="A43" s="17" t="n">
         <v>47</v>
       </c>
-      <c r="B43" s="18" t="n">
+      <c r="B43" s="23" t="n">
         <v>46042</v>
       </c>
       <c r="C43" s="17" t="inlineStr">
@@ -3726,7 +3731,7 @@
       <c r="A44" s="17" t="n">
         <v>48</v>
       </c>
-      <c r="B44" s="18" t="n">
+      <c r="B44" s="23" t="n">
         <v>46042</v>
       </c>
       <c r="C44" s="17" t="inlineStr">
@@ -3766,7 +3771,7 @@
       <c r="A45" s="17" t="n">
         <v>49</v>
       </c>
-      <c r="B45" s="18" t="n">
+      <c r="B45" s="23" t="n">
         <v>46042</v>
       </c>
       <c r="C45" s="17" t="inlineStr">
@@ -3806,7 +3811,7 @@
       <c r="A46" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="B46" s="10" t="n">
+      <c r="B46" s="21" t="n">
         <v>46042</v>
       </c>
       <c r="C46" s="9" t="inlineStr">
@@ -3848,7 +3853,7 @@
       <c r="A47" s="9" t="n">
         <v>51</v>
       </c>
-      <c r="B47" s="10" t="n">
+      <c r="B47" s="21" t="n">
         <v>46042</v>
       </c>
       <c r="C47" s="9" t="inlineStr">
@@ -3888,7 +3893,7 @@
       <c r="A48" s="9" t="n">
         <v>52</v>
       </c>
-      <c r="B48" s="10" t="n">
+      <c r="B48" s="21" t="n">
         <v>46042</v>
       </c>
       <c r="C48" s="9" t="inlineStr">
@@ -3928,7 +3933,7 @@
       <c r="A49" s="17" t="n">
         <v>53</v>
       </c>
-      <c r="B49" s="18" t="n">
+      <c r="B49" s="23" t="n">
         <v>46060</v>
       </c>
       <c r="C49" s="17" t="inlineStr">
@@ -3970,7 +3975,7 @@
       <c r="A50" s="17" t="n">
         <v>54</v>
       </c>
-      <c r="B50" s="18" t="n">
+      <c r="B50" s="23" t="n">
         <v>46060</v>
       </c>
       <c r="C50" s="17" t="inlineStr">
@@ -4010,7 +4015,7 @@
       <c r="A51" s="17" t="n">
         <v>55</v>
       </c>
-      <c r="B51" s="18" t="n">
+      <c r="B51" s="23" t="n">
         <v>46064</v>
       </c>
       <c r="C51" s="17" t="inlineStr">
@@ -4052,7 +4057,7 @@
       <c r="A52" s="17" t="n">
         <v>56</v>
       </c>
-      <c r="B52" s="18" t="n">
+      <c r="B52" s="23" t="n">
         <v>46064</v>
       </c>
       <c r="C52" s="17" t="inlineStr">
@@ -4092,7 +4097,7 @@
       <c r="A53" s="17" t="n">
         <v>57</v>
       </c>
-      <c r="B53" s="18" t="n">
+      <c r="B53" s="23" t="n">
         <v>46064</v>
       </c>
       <c r="C53" s="17" t="inlineStr">
@@ -4132,7 +4137,7 @@
       <c r="A54" s="17" t="n">
         <v>58</v>
       </c>
-      <c r="B54" s="18" t="n">
+      <c r="B54" s="23" t="n">
         <v>46064</v>
       </c>
       <c r="C54" s="17" t="inlineStr">
@@ -4172,7 +4177,7 @@
       <c r="A55" s="17" t="n">
         <v>59</v>
       </c>
-      <c r="B55" s="18" t="n">
+      <c r="B55" s="23" t="n">
         <v>46064</v>
       </c>
       <c r="C55" s="17" t="inlineStr">
@@ -4212,7 +4217,7 @@
       <c r="A56" s="17" t="n">
         <v>60</v>
       </c>
-      <c r="B56" s="18" t="n">
+      <c r="B56" s="23" t="n">
         <v>46064</v>
       </c>
       <c r="C56" s="17" t="inlineStr">
@@ -4252,7 +4257,7 @@
       <c r="A57" s="17" t="n">
         <v>61</v>
       </c>
-      <c r="B57" s="18" t="n">
+      <c r="B57" s="23" t="n">
         <v>46068</v>
       </c>
       <c r="C57" s="17" t="inlineStr">
@@ -4294,7 +4299,7 @@
       <c r="A58" s="17" t="n">
         <v>62</v>
       </c>
-      <c r="B58" s="18" t="n">
+      <c r="B58" s="23" t="n">
         <v>46068</v>
       </c>
       <c r="C58" s="17" t="inlineStr">
@@ -4334,7 +4339,7 @@
       <c r="A59" s="17" t="n">
         <v>63</v>
       </c>
-      <c r="B59" s="18" t="n">
+      <c r="B59" s="23" t="n">
         <v>46068</v>
       </c>
       <c r="C59" s="17" t="inlineStr">
@@ -4374,7 +4379,7 @@
       <c r="A60" s="17" t="n">
         <v>64</v>
       </c>
-      <c r="B60" s="18" t="n">
+      <c r="B60" s="23" t="n">
         <v>46068</v>
       </c>
       <c r="C60" s="17" t="inlineStr">
@@ -4414,7 +4419,7 @@
       <c r="A61" s="9" t="n">
         <v>65</v>
       </c>
-      <c r="B61" s="10" t="n">
+      <c r="B61" s="21" t="n">
         <v>46104</v>
       </c>
       <c r="C61" s="9" t="inlineStr">
@@ -4460,7 +4465,7 @@
       <c r="A62" s="9" t="n">
         <v>66</v>
       </c>
-      <c r="B62" s="10" t="n">
+      <c r="B62" s="21" t="n">
         <v>46104</v>
       </c>
       <c r="C62" s="9" t="inlineStr">
@@ -4500,7 +4505,7 @@
       <c r="A63" s="9" t="n">
         <v>67</v>
       </c>
-      <c r="B63" s="10" t="n">
+      <c r="B63" s="21" t="n">
         <v>46104</v>
       </c>
       <c r="C63" s="9" t="inlineStr">
@@ -4540,7 +4545,7 @@
       <c r="A64" s="17" t="n">
         <v>68</v>
       </c>
-      <c r="B64" s="18" t="n">
+      <c r="B64" s="23" t="n">
         <v>46120</v>
       </c>
       <c r="C64" s="17" t="inlineStr">
@@ -4582,7 +4587,7 @@
       <c r="A65" s="17" t="n">
         <v>69</v>
       </c>
-      <c r="B65" s="18" t="n">
+      <c r="B65" s="23" t="n">
         <v>46121</v>
       </c>
       <c r="C65" s="17" t="inlineStr">
@@ -4624,7 +4629,7 @@
       <c r="A66" s="17" t="n">
         <v>70</v>
       </c>
-      <c r="B66" s="18" t="n">
+      <c r="B66" s="23" t="n">
         <v>46121</v>
       </c>
       <c r="C66" s="17" t="inlineStr">
@@ -4664,7 +4669,7 @@
       <c r="A67" s="17" t="n">
         <v>71</v>
       </c>
-      <c r="B67" s="18" t="n">
+      <c r="B67" s="23" t="n">
         <v>46121</v>
       </c>
       <c r="C67" s="17" t="inlineStr">
@@ -4706,7 +4711,7 @@
       <c r="A68" s="17" t="n">
         <v>72</v>
       </c>
-      <c r="B68" s="18" t="n">
+      <c r="B68" s="23" t="n">
         <v>46121</v>
       </c>
       <c r="C68" s="17" t="inlineStr">
@@ -4746,7 +4751,7 @@
       <c r="A69" s="17" t="n">
         <v>73</v>
       </c>
-      <c r="B69" s="18" t="n">
+      <c r="B69" s="23" t="n">
         <v>46123</v>
       </c>
       <c r="C69" s="17" t="inlineStr">
@@ -4788,7 +4793,7 @@
       <c r="A70" s="17" t="n">
         <v>74</v>
       </c>
-      <c r="B70" s="18" t="n">
+      <c r="B70" s="23" t="n">
         <v>46123</v>
       </c>
       <c r="C70" s="17" t="inlineStr">
@@ -4828,7 +4833,7 @@
       <c r="A71" s="17" t="n">
         <v>75</v>
       </c>
-      <c r="B71" s="18" t="n">
+      <c r="B71" s="23" t="n">
         <v>46127</v>
       </c>
       <c r="C71" s="17" t="inlineStr">
@@ -4870,7 +4875,7 @@
       <c r="A72" s="17" t="n">
         <v>76</v>
       </c>
-      <c r="B72" s="18" t="n">
+      <c r="B72" s="23" t="n">
         <v>46138</v>
       </c>
       <c r="C72" s="17" t="inlineStr">
@@ -4912,7 +4917,7 @@
       <c r="A73" s="17" t="n">
         <v>77</v>
       </c>
-      <c r="B73" s="18" t="n">
+      <c r="B73" s="23" t="n">
         <v>46138</v>
       </c>
       <c r="C73" s="17" t="inlineStr">
@@ -4952,7 +4957,7 @@
       <c r="A74" s="17" t="n">
         <v>78</v>
       </c>
-      <c r="B74" s="18" t="n">
+      <c r="B74" s="23" t="n">
         <v>46144</v>
       </c>
       <c r="C74" s="17" t="inlineStr">
@@ -4994,7 +4999,7 @@
       <c r="A75" s="17" t="n">
         <v>79</v>
       </c>
-      <c r="B75" s="18" t="n">
+      <c r="B75" s="23" t="n">
         <v>46144</v>
       </c>
       <c r="C75" s="17" t="inlineStr">
@@ -5034,7 +5039,7 @@
       <c r="A76" s="17" t="n">
         <v>80</v>
       </c>
-      <c r="B76" s="18" t="n">
+      <c r="B76" s="23" t="n">
         <v>46147</v>
       </c>
       <c r="C76" s="17" t="inlineStr">
@@ -5076,7 +5081,7 @@
       <c r="A77" s="17" t="n">
         <v>81</v>
       </c>
-      <c r="B77" s="18" t="n">
+      <c r="B77" s="23" t="n">
         <v>46147</v>
       </c>
       <c r="C77" s="17" t="inlineStr">
@@ -5116,7 +5121,7 @@
       <c r="A78" s="17" t="n">
         <v>82</v>
       </c>
-      <c r="B78" s="18" t="n">
+      <c r="B78" s="23" t="n">
         <v>46160</v>
       </c>
       <c r="C78" s="17" t="inlineStr">
@@ -5158,7 +5163,7 @@
       <c r="A79" s="17" t="n">
         <v>83</v>
       </c>
-      <c r="B79" s="18" t="n">
+      <c r="B79" s="23" t="n">
         <v>46163</v>
       </c>
       <c r="C79" s="17" t="inlineStr">
@@ -5200,7 +5205,7 @@
       <c r="A80" s="17" t="n">
         <v>84</v>
       </c>
-      <c r="B80" s="18" t="n">
+      <c r="B80" s="23" t="n">
         <v>46163</v>
       </c>
       <c r="C80" s="17" t="inlineStr">
@@ -5240,7 +5245,7 @@
       <c r="A81" s="17" t="n">
         <v>85</v>
       </c>
-      <c r="B81" s="18" t="n">
+      <c r="B81" s="23" t="n">
         <v>46184</v>
       </c>
       <c r="C81" s="17" t="inlineStr">
@@ -5282,7 +5287,7 @@
       <c r="A82" s="17" t="n">
         <v>86</v>
       </c>
-      <c r="B82" s="18" t="n">
+      <c r="B82" s="23" t="n">
         <v>46184</v>
       </c>
       <c r="C82" s="17" t="inlineStr">
@@ -5324,7 +5329,7 @@
       <c r="A83" s="17" t="n">
         <v>87</v>
       </c>
-      <c r="B83" s="18" t="n">
+      <c r="B83" s="23" t="n">
         <v>46184</v>
       </c>
       <c r="C83" s="17" t="inlineStr">
@@ -5364,7 +5369,7 @@
       <c r="A84" s="17" t="n">
         <v>88</v>
       </c>
-      <c r="B84" s="18" t="n">
+      <c r="B84" s="23" t="n">
         <v>46184</v>
       </c>
       <c r="C84" s="17" t="inlineStr">
@@ -5404,7 +5409,7 @@
       <c r="A85" s="9" t="n">
         <v>89</v>
       </c>
-      <c r="B85" s="10" t="n">
+      <c r="B85" s="21" t="n">
         <v>46184</v>
       </c>
       <c r="C85" s="9" t="inlineStr">
@@ -5447,216 +5452,216 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="12" t="n">
+      <c r="A86" s="9" t="n">
         <v>90</v>
       </c>
-      <c r="B86" s="13" t="n">
+      <c r="B86" s="21" t="n">
         <v>46187</v>
       </c>
-      <c r="C86" s="12" t="inlineStr">
+      <c r="C86" s="9" t="inlineStr">
         <is>
           <t>NS-0755</t>
         </is>
       </c>
-      <c r="D86" s="12" t="inlineStr">
+      <c r="D86" s="9" t="inlineStr">
         <is>
           <t>زهور فينكا روزا</t>
         </is>
       </c>
-      <c r="E86" s="12" t="n">
+      <c r="E86" s="9" t="n">
         <v>3500</v>
       </c>
-      <c r="F86" s="12" t="n">
+      <c r="F86" s="9" t="n">
         <v>0.5</v>
       </c>
-      <c r="G86" s="14">
+      <c r="G86" s="11">
         <f>E86*F86</f>
         <v/>
       </c>
-      <c r="H86" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I86" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J86" s="12" t="inlineStr">
-        <is>
-          <t>غير موجود بالنظام</t>
-        </is>
-      </c>
-      <c r="K86" s="12" t="inlineStr">
+      <c r="H86" s="9" t="inlineStr">
+        <is>
+          <t>ISV-0010، ISV-0038</t>
+        </is>
+      </c>
+      <c r="I86" s="9" t="n">
+        <v>7005</v>
+      </c>
+      <c r="J86" s="9" t="inlineStr">
+        <is>
+          <t>يوجد فرق</t>
+        </is>
+      </c>
+      <c r="K86" s="9" t="inlineStr">
         <is>
           <t>يقابله ISV-0010 (14-6) و ISV-0038 (24-6 – جهنمية كبير 5). ⚠ المحاسب أسقط بند رويليا × 94 الموجود بالسند ISV-0010. نفس رقم الطلب NS-0755 استُخدم لتاريخين</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="12" t="n">
+      <c r="A87" s="9" t="n">
         <v>91</v>
       </c>
-      <c r="B87" s="13" t="n">
+      <c r="B87" s="21" t="n">
         <v>46187</v>
       </c>
-      <c r="C87" s="12" t="inlineStr">
+      <c r="C87" s="9" t="inlineStr">
         <is>
           <t>NS-0755</t>
         </is>
       </c>
-      <c r="D87" s="12" t="inlineStr">
+      <c r="D87" s="9" t="inlineStr">
         <is>
           <t>زهور زينيا</t>
         </is>
       </c>
-      <c r="E87" s="12" t="n">
+      <c r="E87" s="9" t="n">
         <v>3500</v>
       </c>
-      <c r="F87" s="12" t="n">
+      <c r="F87" s="9" t="n">
         <v>0.5</v>
       </c>
-      <c r="G87" s="14">
+      <c r="G87" s="11">
         <f>E87*F87</f>
         <v/>
       </c>
-      <c r="H87" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I87" s="12" t="n"/>
-      <c r="J87" s="12" t="inlineStr">
-        <is>
-          <t>غير موجود بالنظام</t>
-        </is>
-      </c>
-      <c r="K87" s="12" t="inlineStr"/>
+      <c r="H87" s="9" t="inlineStr">
+        <is>
+          <t>ISV-0010، ISV-0038</t>
+        </is>
+      </c>
+      <c r="I87" s="9" t="n"/>
+      <c r="J87" s="9" t="inlineStr">
+        <is>
+          <t>يوجد فرق</t>
+        </is>
+      </c>
+      <c r="K87" s="9" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="12" t="n">
+      <c r="A88" s="9" t="n">
         <v>92</v>
       </c>
-      <c r="B88" s="13" t="n">
+      <c r="B88" s="21" t="n">
         <v>46187</v>
       </c>
-      <c r="C88" s="12" t="inlineStr">
+      <c r="C88" s="9" t="inlineStr">
         <is>
           <t>NS-0755</t>
         </is>
       </c>
-      <c r="D88" s="12" t="inlineStr">
+      <c r="D88" s="9" t="inlineStr">
         <is>
           <t>اكاسيا جلوكا من 1 - 2 متر</t>
         </is>
       </c>
-      <c r="E88" s="12" t="n">
+      <c r="E88" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="F88" s="12" t="n">
+      <c r="F88" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="G88" s="14">
+      <c r="G88" s="11">
         <f>E88*F88</f>
         <v/>
       </c>
-      <c r="H88" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I88" s="12" t="n"/>
-      <c r="J88" s="12" t="inlineStr">
-        <is>
-          <t>غير موجود بالنظام</t>
-        </is>
-      </c>
-      <c r="K88" s="12" t="inlineStr"/>
+      <c r="H88" s="9" t="inlineStr">
+        <is>
+          <t>ISV-0010، ISV-0038</t>
+        </is>
+      </c>
+      <c r="I88" s="9" t="n"/>
+      <c r="J88" s="9" t="inlineStr">
+        <is>
+          <t>يوجد فرق</t>
+        </is>
+      </c>
+      <c r="K88" s="9" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="12" t="n">
+      <c r="A89" s="9" t="n">
         <v>93</v>
       </c>
-      <c r="B89" s="13" t="n">
+      <c r="B89" s="21" t="n">
         <v>46187</v>
       </c>
-      <c r="C89" s="12" t="inlineStr">
+      <c r="C89" s="9" t="inlineStr">
         <is>
           <t>NS-0755</t>
         </is>
       </c>
-      <c r="D89" s="12" t="inlineStr">
+      <c r="D89" s="9" t="inlineStr">
         <is>
           <t>كف مريم 1.5 : 2 م</t>
         </is>
       </c>
-      <c r="E89" s="12" t="n">
+      <c r="E89" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="F89" s="12" t="n">
+      <c r="F89" s="9" t="n">
         <v>5.5</v>
       </c>
-      <c r="G89" s="14">
+      <c r="G89" s="11">
         <f>E89*F89</f>
         <v/>
       </c>
-      <c r="H89" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I89" s="12" t="n"/>
-      <c r="J89" s="12" t="inlineStr">
-        <is>
-          <t>غير موجود بالنظام</t>
-        </is>
-      </c>
-      <c r="K89" s="12" t="inlineStr"/>
+      <c r="H89" s="9" t="inlineStr">
+        <is>
+          <t>ISV-0010، ISV-0038</t>
+        </is>
+      </c>
+      <c r="I89" s="9" t="n"/>
+      <c r="J89" s="9" t="inlineStr">
+        <is>
+          <t>يوجد فرق</t>
+        </is>
+      </c>
+      <c r="K89" s="9" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="12" t="n">
+      <c r="A90" s="9" t="n">
         <v>97</v>
       </c>
-      <c r="B90" s="13" t="n">
+      <c r="B90" s="21" t="n">
         <v>46197</v>
       </c>
-      <c r="C90" s="12" t="inlineStr">
+      <c r="C90" s="9" t="inlineStr">
         <is>
           <t>NS-0755</t>
         </is>
       </c>
-      <c r="D90" s="12" t="inlineStr">
+      <c r="D90" s="9" t="inlineStr">
         <is>
           <t>جهنمية كروية تايلندي كبير</t>
         </is>
       </c>
-      <c r="E90" s="12" t="n">
+      <c r="E90" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="F90" s="12" t="n">
+      <c r="F90" s="9" t="n">
         <v>300</v>
       </c>
-      <c r="G90" s="14">
+      <c r="G90" s="11">
         <f>E90*F90</f>
         <v/>
       </c>
-      <c r="H90" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I90" s="12" t="n"/>
-      <c r="J90" s="12" t="inlineStr">
-        <is>
-          <t>غير موجود بالنظام</t>
-        </is>
-      </c>
-      <c r="K90" s="12" t="inlineStr"/>
+      <c r="H90" s="9" t="inlineStr">
+        <is>
+          <t>ISV-0010، ISV-0038</t>
+        </is>
+      </c>
+      <c r="I90" s="9" t="n"/>
+      <c r="J90" s="9" t="inlineStr">
+        <is>
+          <t>يوجد فرق</t>
+        </is>
+      </c>
+      <c r="K90" s="9" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="17" t="n">
         <v>94</v>
       </c>
-      <c r="B91" s="18" t="n">
+      <c r="B91" s="23" t="n">
         <v>46187</v>
       </c>
       <c r="C91" s="17" t="inlineStr">
@@ -5702,7 +5707,7 @@
       <c r="A92" s="17" t="n">
         <v>95</v>
       </c>
-      <c r="B92" s="18" t="n">
+      <c r="B92" s="23" t="n">
         <v>46190</v>
       </c>
       <c r="C92" s="17" t="inlineStr">
@@ -5744,7 +5749,7 @@
       <c r="A93" s="17" t="n">
         <v>96</v>
       </c>
-      <c r="B93" s="18" t="n">
+      <c r="B93" s="23" t="n">
         <v>46195</v>
       </c>
       <c r="C93" s="17" t="inlineStr">
@@ -5786,7 +5791,7 @@
       <c r="A94" s="17" t="n">
         <v>98</v>
       </c>
-      <c r="B94" s="18" t="n">
+      <c r="B94" s="23" t="n">
         <v>46200</v>
       </c>
       <c r="C94" s="17" t="inlineStr">
@@ -5828,7 +5833,7 @@
       <c r="A95" s="17" t="n">
         <v>99</v>
       </c>
-      <c r="B95" s="18" t="n">
+      <c r="B95" s="23" t="n">
         <v>46201</v>
       </c>
       <c r="C95" s="17" t="inlineStr">
@@ -5870,7 +5875,7 @@
       <c r="A96" s="17" t="n">
         <v>100</v>
       </c>
-      <c r="B96" s="18" t="n">
+      <c r="B96" s="23" t="n">
         <v>46205</v>
       </c>
       <c r="C96" s="17" t="inlineStr">
@@ -5912,7 +5917,7 @@
       <c r="A97" s="9" t="n">
         <v>101</v>
       </c>
-      <c r="B97" s="10" t="n">
+      <c r="B97" s="21" t="n">
         <v>46209</v>
       </c>
       <c r="C97" s="9" t="inlineStr">
@@ -5958,7 +5963,7 @@
       <c r="A98" s="9" t="n">
         <v>102</v>
       </c>
-      <c r="B98" s="10" t="n">
+      <c r="B98" s="21" t="n">
         <v>46209</v>
       </c>
       <c r="C98" s="9" t="inlineStr">
@@ -5998,7 +6003,7 @@
       <c r="A99" s="9" t="n">
         <v>103</v>
       </c>
-      <c r="B99" s="10" t="n">
+      <c r="B99" s="21" t="n">
         <v>46209</v>
       </c>
       <c r="C99" s="9" t="inlineStr">
@@ -6038,7 +6043,7 @@
       <c r="A100" s="17" t="n">
         <v>104</v>
       </c>
-      <c r="B100" s="18" t="n">
+      <c r="B100" s="23" t="n">
         <v>46214</v>
       </c>
       <c r="C100" s="17" t="inlineStr">
@@ -6080,7 +6085,7 @@
       <c r="A101" s="17" t="n">
         <v>105</v>
       </c>
-      <c r="B101" s="18" t="n">
+      <c r="B101" s="23" t="n">
         <v>46214</v>
       </c>
       <c r="C101" s="17" t="inlineStr">
@@ -6122,7 +6127,7 @@
       <c r="A102" s="17" t="n">
         <v>106</v>
       </c>
-      <c r="B102" s="18" t="n">
+      <c r="B102" s="23" t="n">
         <v>46214</v>
       </c>
       <c r="C102" s="17" t="inlineStr">
@@ -6164,7 +6169,7 @@
       <c r="A103" s="9" t="n">
         <v>107</v>
       </c>
-      <c r="B103" s="10" t="n">
+      <c r="B103" s="21" t="n">
         <v>46214</v>
       </c>
       <c r="C103" s="9" t="inlineStr">
@@ -6208,7 +6213,7 @@
       <c r="A104" s="9" t="n">
         <v>108</v>
       </c>
-      <c r="B104" s="10" t="n">
+      <c r="B104" s="21" t="n">
         <v>46214</v>
       </c>
       <c r="C104" s="9" t="inlineStr">
@@ -6248,7 +6253,7 @@
       <c r="A105" s="9" t="n">
         <v>109</v>
       </c>
-      <c r="B105" s="10" t="n">
+      <c r="B105" s="21" t="n">
         <v>46214</v>
       </c>
       <c r="C105" s="9" t="inlineStr">
@@ -6288,7 +6293,7 @@
       <c r="A106" s="17" t="n">
         <v>110</v>
       </c>
-      <c r="B106" s="18" t="n">
+      <c r="B106" s="23" t="n">
         <v>46229</v>
       </c>
       <c r="C106" s="17" t="inlineStr">
@@ -6330,7 +6335,7 @@
       <c r="A107" s="17" t="n">
         <v>111</v>
       </c>
-      <c r="B107" s="18" t="n">
+      <c r="B107" s="23" t="n">
         <v>46229</v>
       </c>
       <c r="C107" s="17" t="inlineStr">
@@ -6372,7 +6377,7 @@
       <c r="A108" s="17" t="n">
         <v>112</v>
       </c>
-      <c r="B108" s="18" t="n">
+      <c r="B108" s="23" t="n">
         <v>46229</v>
       </c>
       <c r="C108" s="17" t="inlineStr">
@@ -6412,7 +6417,7 @@
       <c r="A109" s="17" t="n">
         <v>113</v>
       </c>
-      <c r="B109" s="18" t="n">
+      <c r="B109" s="23" t="n">
         <v>46229</v>
       </c>
       <c r="C109" s="17" t="inlineStr">
@@ -6539,7 +6544,7 @@
           <t>TNR-2689</t>
         </is>
       </c>
-      <c r="C2" s="20" t="n">
+      <c r="C2" s="24" t="n">
         <v>45959</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -6568,7 +6573,7 @@
           <t>TNR-2888</t>
         </is>
       </c>
-      <c r="C3" s="20" t="n">
+      <c r="C3" s="24" t="n">
         <v>45976</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -6597,7 +6602,7 @@
           <t>TRF-0188</t>
         </is>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="24" t="n">
         <v>46231</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -6626,7 +6631,7 @@
           <t>RNT-1789</t>
         </is>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="24" t="n">
         <v>45863</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -6659,7 +6664,7 @@
           <t>RNT-2166</t>
         </is>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="24" t="n">
         <v>45887</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -6688,7 +6693,7 @@
           <t>RNT-2141</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="24" t="n">
         <v>45909</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -6717,7 +6722,7 @@
           <t>RNT-3077</t>
         </is>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="24" t="n">
         <v>45992</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -6746,7 +6751,7 @@
           <t>RNT-3346</t>
         </is>
       </c>
-      <c r="C9" s="20" t="n">
+      <c r="C9" s="24" t="n">
         <v>46016</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -6775,7 +6780,7 @@
           <t>RNP-2297</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="24" t="n">
         <v>45926</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -6804,7 +6809,7 @@
           <t>RNP-2427</t>
         </is>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="24" t="n">
         <v>45938</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -6833,7 +6838,7 @@
           <t>RNP-3756</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="24" t="n">
         <v>46057</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -6862,7 +6867,7 @@
           <t>ISV-0075</t>
         </is>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="24" t="n">
         <v>46207</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -6895,7 +6900,7 @@
           <t>RNP-1787</t>
         </is>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="24" t="n">
         <v>45863</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -6928,7 +6933,7 @@
           <t>RNP-1787</t>
         </is>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="24" t="n">
         <v>45873</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -6961,7 +6966,7 @@
           <t>TRF-0107 (جزء)</t>
         </is>
       </c>
-      <c r="C16" s="20" t="n">
+      <c r="C16" s="24" t="n">
         <v>46214</v>
       </c>
       <c r="D16" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add pre-period Riyadh-to-Tabuk purchase orders sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA2XXv3viuKc4AVC546mfn
</commit_message>
<xml_diff>
--- a/مراجعة_شيتات_المسحوبات_الرياض_تبوك.xlsx
+++ b/مراجعة_شيتات_المسحوبات_الرياض_تبوك.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="ملخص المراجعة" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="مسحوبات الرياض من تبوك" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="مسحوبات تبوك من الرياض" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="سندات بالنظام غير مدرجة" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="مسحوبات قبل الفترة" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="مسحوبات الرياض من تبوك" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="مسحوبات تبوك من الرياض" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="سندات بالنظام غير مدرجة" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,10 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +42,10 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="7">
@@ -101,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -142,6 +148,20 @@
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -772,6 +792,386 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="70" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>مسحوبات تبوك من مزرعة الرياض قبل الفترة المقررة – أوامر شراء (المورد بالمستند: مؤسسة بساتين الرياض)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>الأسعار غير موجودة في المستندات (سعر الوحدة = 0.00) – خانة السعر باللون الأصفر للإدخال اليدوي، والإجمالي يُحسب تلقائياً.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>أمر الشراء</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>مرجع الطلب</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>تاريخ الأمر</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>تاريخ الوصول المتوقع</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>الصنف</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>الكمية</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>سعر الوحدة (يدوي)</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>تكلفة البراد / الإيجار</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>من تحمّل التكلفة</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>ملاحظة المستند</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>P00508</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>49009</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="n">
+        <v>45854</v>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>45854</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>فينكا أحمر</t>
+        </is>
+      </c>
+      <c r="F5" s="26" t="n">
+        <v>6000</v>
+      </c>
+      <c r="G5" s="27" t="n"/>
+      <c r="H5" s="4">
+        <f>F5*G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>3500</v>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>نسما الشرق</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>تم التحميل مع زهور أخرى من البستان ونوّارة، ودفع الإيجار 3,500 عن طريق نسما الشرق</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>P00508</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>49009</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="n">
+        <v>45854</v>
+      </c>
+      <c r="D6" s="24" t="n">
+        <v>45854</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>فينكا أبيض</t>
+        </is>
+      </c>
+      <c r="F6" s="26" t="n">
+        <v>6000</v>
+      </c>
+      <c r="G6" s="27" t="n"/>
+      <c r="H6" s="4">
+        <f>F6*G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="3" t="inlineStr"/>
+      <c r="K6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>P00519</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>47697</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="n">
+        <v>45856</v>
+      </c>
+      <c r="D7" s="24" t="n">
+        <v>45820</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>زهور موسمية (SEASONAL FLOWERS)</t>
+        </is>
+      </c>
+      <c r="F7" s="26" t="n">
+        <v>42000</v>
+      </c>
+      <c r="G7" s="27" t="n"/>
+      <c r="H7" s="4">
+        <f>F7*G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>3800</v>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>نسما الشرق</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>تم حساب البراد عن طريق نسما الشرق 3,800 ريال</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>P00522</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>NS-1466</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="n">
+        <v>45856</v>
+      </c>
+      <c r="D8" s="24" t="n">
+        <v>45837</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>زهور موسمية – غير شامل التوصيل</t>
+        </is>
+      </c>
+      <c r="F8" s="26" t="n">
+        <v>15000</v>
+      </c>
+      <c r="G8" s="27" t="n"/>
+      <c r="H8" s="4">
+        <f>F8*G8</f>
+        <v/>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>نسما الشرق</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>غير شامل التوصيل وغير شامل إيجار البراد 3,000 – تم الحساب من نسما الشرق</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>P00523</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>NS-1314</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="n">
+        <v>45856</v>
+      </c>
+      <c r="D9" s="24" t="n">
+        <v>45820</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>زهور موسمية (SEASONAL FLOWERS)</t>
+        </is>
+      </c>
+      <c r="F9" s="26" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G9" s="27" t="n"/>
+      <c r="H9" s="4">
+        <f>F9*G9</f>
+        <v/>
+      </c>
+      <c r="I9" s="4" t="n"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>جرين تاون</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>تم حساب البراد عن طريق جرين تاون – إجمالي الحمولة 15,000 وتم قبول 9,000 فقط</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr"/>
+      <c r="B10" s="15" t="inlineStr"/>
+      <c r="C10" s="15" t="inlineStr"/>
+      <c r="D10" s="15" t="inlineStr"/>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="F10" s="28">
+        <f>SUM(F5:F9)</f>
+        <v/>
+      </c>
+      <c r="G10" s="15" t="inlineStr"/>
+      <c r="H10" s="16">
+        <f>SUM(H5:H9)</f>
+        <v/>
+      </c>
+      <c r="I10" s="16">
+        <f>SUM(I5:I9)</f>
+        <v/>
+      </c>
+      <c r="J10" s="15" t="n"/>
+      <c r="K10" s="15" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>ملاحظات:</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>1) تواريخ الوصول المتوقع في P00519 و P00522 و P00523 (يونيو 2025) أسبق من تاريخ أمر الشراء (18-7-2025) – يعني الأوامر سُجلت بعد الاستلام.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>2) P00523: الحمولة 15,000 وتم قبول 9,000 فقط – الكمية المدرجة 9,000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>3) تكاليف البراد والإيجار التي تحمّلتها نسما الشرق = 10,300 ريال (3,500 + 3,800 + 3,000)، وتكلفة براد P00523 على جرين تاون.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>4) المورد المذكور بأوامر الشراء "مؤسسة بساتين الرياض". الأصناف في P00519 و P00522 و P00523 مكتوبة "زهور موسمية" بدون تفصيل.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A12:K12"/>
+    <mergeCell ref="A15:K15"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A11:K11"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A13:K13"/>
+    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1926,7 +2326,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6478,7 +6878,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add POs P00480/P00481 to pre-period withdrawals
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA2XXv3viuKc4AVC546mfn
</commit_message>
<xml_diff>
--- a/مراجعة_شيتات_المسحوبات_الرياض_تبوك.xlsx
+++ b/مراجعة_شيتات_المسحوبات_الرياض_تبوك.xlsx
@@ -792,14 +792,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
@@ -865,7 +865,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>تكلفة البراد / الإيجار</t>
+          <t>تكلفة البراد / النقل</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -882,27 +882,27 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>P00508</t>
+          <t>P00480</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>49009</t>
+          <t>45802</t>
         </is>
       </c>
       <c r="C5" s="24" t="n">
-        <v>45854</v>
+        <v>45845</v>
       </c>
       <c r="D5" s="24" t="n">
-        <v>45854</v>
+        <v>45844</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>فينكا أحمر</t>
+          <t>فينكا أبيض نقطة حمراء</t>
         </is>
       </c>
       <c r="F5" s="26" t="n">
-        <v>6000</v>
+        <v>3875</v>
       </c>
       <c r="G5" s="27" t="n"/>
       <c r="H5" s="4">
@@ -910,7 +910,7 @@
         <v/>
       </c>
       <c r="I5" s="4" t="n">
-        <v>3500</v>
+        <v>2800</v>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
@@ -919,34 +919,34 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>تم التحميل مع زهور أخرى من البستان ونوّارة، ودفع الإيجار 3,500 عن طريق نسما الشرق</t>
+          <t>تم دفع إيجار النقل عن طريق نسما الشرق للتعميد رقم 480 - 481 مبلغ 2,800 ريال (مبلغ واحد للأمرين)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>P00508</t>
+          <t>P00480</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>49009</t>
+          <t>45802</t>
         </is>
       </c>
       <c r="C6" s="24" t="n">
-        <v>45854</v>
+        <v>45845</v>
       </c>
       <c r="D6" s="24" t="n">
-        <v>45854</v>
+        <v>45844</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>فينكا أبيض</t>
+          <t>فينكا أحمر بنقطة</t>
         </is>
       </c>
       <c r="F6" s="26" t="n">
-        <v>6000</v>
+        <v>3000</v>
       </c>
       <c r="G6" s="27" t="n"/>
       <c r="H6" s="4">
@@ -960,36 +960,34 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>P00519</t>
+          <t>P00481</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>47697</t>
+          <t>NS-1466</t>
         </is>
       </c>
       <c r="C7" s="24" t="n">
-        <v>45856</v>
+        <v>45845</v>
       </c>
       <c r="D7" s="24" t="n">
-        <v>45820</v>
+        <v>45844</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>زهور موسمية (SEASONAL FLOWERS)</t>
+          <t>فينكا أحمر</t>
         </is>
       </c>
       <c r="F7" s="26" t="n">
-        <v>42000</v>
+        <v>5000</v>
       </c>
       <c r="G7" s="27" t="n"/>
       <c r="H7" s="4">
         <f>F7*G7</f>
         <v/>
       </c>
-      <c r="I7" s="4" t="n">
-        <v>3800</v>
-      </c>
+      <c r="I7" s="4" t="n"/>
       <c r="J7" s="3" t="inlineStr">
         <is>
           <t>نسما الشرق</t>
@@ -997,14 +995,14 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>تم حساب البراد عن طريق نسما الشرق 3,800 ريال</t>
+          <t>ضمن مبلغ النقل 2,800 المشترك مع P00480</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>P00522</t>
+          <t>P00481</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1013,62 +1011,52 @@
         </is>
       </c>
       <c r="C8" s="24" t="n">
-        <v>45856</v>
+        <v>45845</v>
       </c>
       <c r="D8" s="24" t="n">
-        <v>45837</v>
+        <v>45844</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>زهور موسمية – غير شامل التوصيل</t>
+          <t>فينكا أزرق</t>
         </is>
       </c>
       <c r="F8" s="26" t="n">
-        <v>15000</v>
+        <v>5000</v>
       </c>
       <c r="G8" s="27" t="n"/>
       <c r="H8" s="4">
         <f>F8*G8</f>
         <v/>
       </c>
-      <c r="I8" s="4" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>نسما الشرق</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>غير شامل التوصيل وغير شامل إيجار البراد 3,000 – تم الحساب من نسما الشرق</t>
-        </is>
-      </c>
+      <c r="I8" s="4" t="n"/>
+      <c r="J8" s="3" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>P00523</t>
+          <t>P00481</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>NS-1314</t>
+          <t>NS-1466</t>
         </is>
       </c>
       <c r="C9" s="24" t="n">
-        <v>45856</v>
+        <v>45845</v>
       </c>
       <c r="D9" s="24" t="n">
-        <v>45820</v>
+        <v>45844</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>زهور موسمية (SEASONAL FLOWERS)</t>
+          <t>فينكا أبيض</t>
         </is>
       </c>
       <c r="F9" s="26" t="n">
-        <v>9000</v>
+        <v>3000</v>
       </c>
       <c r="G9" s="27" t="n"/>
       <c r="H9" s="4">
@@ -1076,91 +1064,341 @@
         <v/>
       </c>
       <c r="I9" s="4" t="n"/>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>P00481</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>NS-1466</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="n">
+        <v>45845</v>
+      </c>
+      <c r="D10" s="24" t="n">
+        <v>45844</v>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>فينكا مشمشي</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G10" s="27" t="n"/>
+      <c r="H10" s="4">
+        <f>F10*G10</f>
+        <v/>
+      </c>
+      <c r="I10" s="4" t="n"/>
+      <c r="J10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>P00508</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>49009</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="n">
+        <v>45854</v>
+      </c>
+      <c r="D11" s="24" t="n">
+        <v>45854</v>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>فينكا أحمر</t>
+        </is>
+      </c>
+      <c r="F11" s="26" t="n">
+        <v>6000</v>
+      </c>
+      <c r="G11" s="27" t="n"/>
+      <c r="H11" s="4">
+        <f>F11*G11</f>
+        <v/>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>3500</v>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>نسما الشرق</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>تم التحميل مع زهور أخرى من البستان ونوّارة، ودفع الإيجار 3,500 عن طريق نسما الشرق</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>P00508</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>49009</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="n">
+        <v>45854</v>
+      </c>
+      <c r="D12" s="24" t="n">
+        <v>45854</v>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>فينكا أبيض</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="n">
+        <v>6000</v>
+      </c>
+      <c r="G12" s="27" t="n"/>
+      <c r="H12" s="4">
+        <f>F12*G12</f>
+        <v/>
+      </c>
+      <c r="I12" s="4" t="n"/>
+      <c r="J12" s="3" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>P00519</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>47697</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="n">
+        <v>45856</v>
+      </c>
+      <c r="D13" s="24" t="n">
+        <v>45820</v>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>زهور موسمية (SEASONAL FLOWERS)</t>
+        </is>
+      </c>
+      <c r="F13" s="26" t="n">
+        <v>42000</v>
+      </c>
+      <c r="G13" s="27" t="n"/>
+      <c r="H13" s="4">
+        <f>F13*G13</f>
+        <v/>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>3800</v>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>نسما الشرق</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>تم حساب البراد عن طريق نسما الشرق 3,800 ريال</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>P00522</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NS-1466</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="n">
+        <v>45856</v>
+      </c>
+      <c r="D14" s="24" t="n">
+        <v>45837</v>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>زهور موسمية – غير شامل التوصيل</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="n">
+        <v>15000</v>
+      </c>
+      <c r="G14" s="27" t="n"/>
+      <c r="H14" s="4">
+        <f>F14*G14</f>
+        <v/>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>نسما الشرق</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>غير شامل التوصيل وغير شامل إيجار البراد 3,000 – تم الحساب من نسما الشرق</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>P00523</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>NS-1314</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="n">
+        <v>45856</v>
+      </c>
+      <c r="D15" s="24" t="n">
+        <v>45820</v>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>زهور موسمية (SEASONAL FLOWERS)</t>
+        </is>
+      </c>
+      <c r="F15" s="26" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G15" s="27" t="n"/>
+      <c r="H15" s="4">
+        <f>F15*G15</f>
+        <v/>
+      </c>
+      <c r="I15" s="4" t="n"/>
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>جرين تاون</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K15" s="3" t="inlineStr">
         <is>
           <t>تم حساب البراد عن طريق جرين تاون – إجمالي الحمولة 15,000 وتم قبول 9,000 فقط</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="15" t="inlineStr"/>
-      <c r="B10" s="15" t="inlineStr"/>
-      <c r="C10" s="15" t="inlineStr"/>
-      <c r="D10" s="15" t="inlineStr"/>
-      <c r="E10" s="15" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr"/>
+      <c r="B16" s="15" t="inlineStr"/>
+      <c r="C16" s="15" t="inlineStr"/>
+      <c r="D16" s="15" t="inlineStr"/>
+      <c r="E16" s="15" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="F10" s="28">
-        <f>SUM(F5:F9)</f>
-        <v/>
-      </c>
-      <c r="G10" s="15" t="inlineStr"/>
-      <c r="H10" s="16">
-        <f>SUM(H5:H9)</f>
-        <v/>
-      </c>
-      <c r="I10" s="16">
-        <f>SUM(I5:I9)</f>
-        <v/>
-      </c>
-      <c r="J10" s="15" t="n"/>
-      <c r="K10" s="15" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="29" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="F16" s="28">
+        <f>SUM(F5:F15)</f>
+        <v/>
+      </c>
+      <c r="G16" s="15" t="inlineStr"/>
+      <c r="H16" s="16">
+        <f>SUM(H5:H15)</f>
+        <v/>
+      </c>
+      <c r="I16" s="16">
+        <f>SUM(I5:I15)</f>
+        <v/>
+      </c>
+      <c r="J16" s="15" t="n"/>
+      <c r="K16" s="15" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>ملاحظات:</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="29" t="inlineStr">
-        <is>
-          <t>1) تواريخ الوصول المتوقع في P00519 و P00522 و P00523 (يونيو 2025) أسبق من تاريخ أمر الشراء (18-7-2025) – يعني الأوامر سُجلت بعد الاستلام.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="29" t="inlineStr">
-        <is>
-          <t>2) P00523: الحمولة 15,000 وتم قبول 9,000 فقط – الكمية المدرجة 9,000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="29" t="inlineStr">
-        <is>
-          <t>3) تكاليف البراد والإيجار التي تحمّلتها نسما الشرق = 10,300 ريال (3,500 + 3,800 + 3,000)، وتكلفة براد P00523 على جرين تاون.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="29" t="inlineStr">
-        <is>
-          <t>4) المورد المذكور بأوامر الشراء "مؤسسة بساتين الرياض". الأصناف في P00519 و P00522 و P00523 مكتوبة "زهور موسمية" بدون تفصيل.</t>
+    <row r="19">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>1) P00480 و P00481 (7-7-2025): مبلغ نقل واحد 2,800 ريال للأمرين دفعته نسما الشرق.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>2) ⚠ مرجع الطلب NS-1466 مستخدم في أمرين مختلفين: P00481 (7-7-2025، فينكا 18,000) و P00522 (18-7-2025، زهور موسمية 15,000) – يلزم التأكد أنهما شحنتان مختلفتان.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>3) تواريخ الوصول المتوقع في P00519 و P00522 و P00523 (يونيو 2025) أسبق من تاريخ أمر الشراء (18-7-2025) – الأوامر سُجلت بعد الاستلام.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="29" t="inlineStr">
+        <is>
+          <t>4) P00523: الحمولة 15,000 وتم قبول 9,000 فقط – الكمية المدرجة 9,000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="29" t="inlineStr">
+        <is>
+          <t>5) تكاليف النقل والبراد التي تحمّلتها نسما الشرق = 13,100 ريال (2,800 + 3,500 + 3,800 + 3,000)، وتكلفة براد P00523 على جرين تاون.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>6) المورد المذكور بأوامر الشراء "مؤسسة بساتين الرياض". الأصناف في P00519 و P00522 و P00523 مكتوبة "زهور موسمية" بدون تفصيل.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A12:K12"/>
-    <mergeCell ref="A15:K15"/>
+  <mergeCells count="10">
+    <mergeCell ref="A22:K22"/>
+    <mergeCell ref="A18:K18"/>
+    <mergeCell ref="A20:K20"/>
+    <mergeCell ref="A21:K21"/>
+    <mergeCell ref="A23:K23"/>
+    <mergeCell ref="A24:K24"/>
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A11:K11"/>
-    <mergeCell ref="A16:K16"/>
-    <mergeCell ref="A13:K13"/>
-    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="A19:K19"/>
     <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A17:K17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add admin expenses and diesel paid by Tabuk for Riyadh farm
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA2XXv3viuKc4AVC546mfn
</commit_message>
<xml_diff>
--- a/مراجعة_شيتات_المسحوبات_الرياض_تبوك.xlsx
+++ b/مراجعة_شيتات_المسحوبات_الرياض_تبوك.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet name="ملخص المراجعة" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="مسحوبات قبل الفترة" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="مسحوبات الرياض من تبوك" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="مسحوبات تبوك من الرياض" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="سندات بالنظام غير مدرجة" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="مصاريف إدارية ووقود من تبوك" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="مسحوبات الرياض من تبوك" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="مسحوبات تبوك من الرياض" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="سندات بالنظام غير مدرجة" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,8 +48,13 @@
       <b val="1"/>
       <sz val="13"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -80,6 +86,11 @@
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -107,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -163,6 +174,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1410,6 +1429,1008 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>المصاريف الإدارية والوقود المدفوعة لمزرعة الرياض عن طريق مزرعة تبوك (نسما الشرق) – عامي 2025 و 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="31" t="inlineStr">
+        <is>
+          <t>أولاً: المصاريف الإدارية 2025 (المصدر: كشف المصاريف الإدارية – البنود 49 إلى 55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B4" s="32" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="C4" s="32" t="inlineStr">
+        <is>
+          <t>البيان</t>
+        </is>
+      </c>
+      <c r="D4" s="32" t="inlineStr">
+        <is>
+          <t>المبلغ</t>
+        </is>
+      </c>
+      <c r="E4" s="32" t="inlineStr">
+        <is>
+          <t>التصنيف</t>
+        </is>
+      </c>
+      <c r="F4" s="32" t="inlineStr">
+        <is>
+          <t>ملاحظة</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="33" t="n">
+        <v>49</v>
+      </c>
+      <c r="B5" s="33" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C5" s="33" t="inlineStr">
+        <is>
+          <t>رسوم تأشيرة مهندس محمد</t>
+        </is>
+      </c>
+      <c r="D5" s="34" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E5" s="33" t="inlineStr">
+        <is>
+          <t>مصاريف إدارية</t>
+        </is>
+      </c>
+      <c r="F5" s="33" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="33" t="n">
+        <v>50</v>
+      </c>
+      <c r="B6" s="33" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="inlineStr">
+        <is>
+          <t>تأشيرة حسين مصطفى المحاسب</t>
+        </is>
+      </c>
+      <c r="D6" s="34" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E6" s="33" t="inlineStr">
+        <is>
+          <t>مصاريف إدارية</t>
+        </is>
+      </c>
+      <c r="F6" s="33" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="33" t="n">
+        <v>51</v>
+      </c>
+      <c r="B7" s="33" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C7" s="33" t="inlineStr">
+        <is>
+          <t>نقل كفالة عظمت</t>
+        </is>
+      </c>
+      <c r="D7" s="34" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E7" s="33" t="inlineStr">
+        <is>
+          <t>مصاريف إدارية</t>
+        </is>
+      </c>
+      <c r="F7" s="33" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="33" t="n">
+        <v>52</v>
+      </c>
+      <c r="B8" s="33" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="inlineStr">
+        <is>
+          <t>نقل كفالة العامل البنجالي 6000 + تجديد إقامة 9 شهور 7925</t>
+        </is>
+      </c>
+      <c r="D8" s="34" t="n">
+        <v>13925</v>
+      </c>
+      <c r="E8" s="33" t="inlineStr">
+        <is>
+          <t>مصاريف إدارية</t>
+        </is>
+      </c>
+      <c r="F8" s="33" t="inlineStr">
+        <is>
+          <t>البند 52 = 6,000 + 7,925 = 13,925 ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="33" t="n">
+        <v>53</v>
+      </c>
+      <c r="B9" s="33" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="inlineStr">
+        <is>
+          <t>تجديد إقامة عظمت عام 2024 + 2025 مع التأمين الطبي</t>
+        </is>
+      </c>
+      <c r="D9" s="34" t="n">
+        <v>20700</v>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
+        <is>
+          <t>مصاريف إدارية</t>
+        </is>
+      </c>
+      <c r="F9" s="33" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="33" t="n">
+        <v>54</v>
+      </c>
+      <c r="B10" s="33" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="inlineStr">
+        <is>
+          <t>تجديد إقامة مهندس محمد عبدالمجيد عام 2025 + التأمين الطبي</t>
+        </is>
+      </c>
+      <c r="D10" s="34" t="n">
+        <v>10650</v>
+      </c>
+      <c r="E10" s="33" t="inlineStr">
+        <is>
+          <t>مصاريف إدارية</t>
+        </is>
+      </c>
+      <c r="F10" s="33" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="33" t="n">
+        <v>55</v>
+      </c>
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="inlineStr">
+        <is>
+          <t>تجديد إقامة حسين مصطفى المحاسب عام 2025 + التأمين الطبي</t>
+        </is>
+      </c>
+      <c r="D11" s="34" t="n">
+        <v>2850</v>
+      </c>
+      <c r="E11" s="33" t="inlineStr">
+        <is>
+          <t>مصاريف إدارية</t>
+        </is>
+      </c>
+      <c r="F11" s="33" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr"/>
+      <c r="B12" s="15" t="inlineStr"/>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>إجمالي المصاريف الإدارية 2025</t>
+        </is>
+      </c>
+      <c r="D12" s="16">
+        <f>SUM(D5:D11)</f>
+        <v/>
+      </c>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="31" t="inlineStr">
+        <is>
+          <t>ثانياً: المصاريف الإدارية والحكومية 2026 (المصدر: تقرير العهدة – Custody Report بتاريخ 9-8-2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="32" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B15" s="32" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="C15" s="32" t="inlineStr">
+        <is>
+          <t>البيان</t>
+        </is>
+      </c>
+      <c r="D15" s="32" t="inlineStr">
+        <is>
+          <t>المبلغ</t>
+        </is>
+      </c>
+      <c r="E15" s="32" t="inlineStr">
+        <is>
+          <t>التصنيف</t>
+        </is>
+      </c>
+      <c r="F15" s="32" t="inlineStr">
+        <is>
+          <t>ملاحظة</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="35" t="n">
+        <v>46160</v>
+      </c>
+      <c r="C16" s="33" t="inlineStr">
+        <is>
+          <t>تجديد إقامة عماد حمدي – 104723160012238</t>
+        </is>
+      </c>
+      <c r="D16" s="34" t="n">
+        <v>2288</v>
+      </c>
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>إقامات ورسوم حكومية</t>
+        </is>
+      </c>
+      <c r="F16" s="33" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="35" t="n">
+        <v>46176</v>
+      </c>
+      <c r="C17" s="33" t="inlineStr">
+        <is>
+          <t>التأمين الطبي لمزرعة الرياض</t>
+        </is>
+      </c>
+      <c r="D17" s="34" t="n">
+        <v>1928.07</v>
+      </c>
+      <c r="E17" s="33" t="inlineStr">
+        <is>
+          <t>تأمين طبي</t>
+        </is>
+      </c>
+      <c r="F17" s="33" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" s="35" t="n">
+        <v>46177</v>
+      </c>
+      <c r="C18" s="33" t="inlineStr">
+        <is>
+          <t>القيمة المضافة تبع تأمين مزرعة الرياض</t>
+        </is>
+      </c>
+      <c r="D18" s="34" t="n">
+        <v>289.21</v>
+      </c>
+      <c r="E18" s="33" t="inlineStr">
+        <is>
+          <t>تأمين طبي</t>
+        </is>
+      </c>
+      <c r="F18" s="33" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="33" t="n">
+        <v>4</v>
+      </c>
+      <c r="B19" s="35" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C19" s="33" t="inlineStr">
+        <is>
+          <t>رخص عمل عصمت الله</t>
+        </is>
+      </c>
+      <c r="D19" s="34" t="n">
+        <v>2425</v>
+      </c>
+      <c r="E19" s="33" t="inlineStr">
+        <is>
+          <t>إقامات ورسوم حكومية</t>
+        </is>
+      </c>
+      <c r="F19" s="33" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="B20" s="35" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C20" s="33" t="inlineStr">
+        <is>
+          <t>رسوم جوازات</t>
+        </is>
+      </c>
+      <c r="D20" s="34" t="n">
+        <v>163</v>
+      </c>
+      <c r="E20" s="33" t="inlineStr">
+        <is>
+          <t>إقامات ورسوم حكومية</t>
+        </is>
+      </c>
+      <c r="F20" s="33" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="B21" s="35" t="n">
+        <v>46191</v>
+      </c>
+      <c r="C21" s="33" t="inlineStr">
+        <is>
+          <t>رخصة عمل حسين مصطفى</t>
+        </is>
+      </c>
+      <c r="D21" s="34" t="n">
+        <v>2425</v>
+      </c>
+      <c r="E21" s="33" t="inlineStr">
+        <is>
+          <t>إقامات ورسوم حكومية</t>
+        </is>
+      </c>
+      <c r="F21" s="33" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="33" t="n">
+        <v>7</v>
+      </c>
+      <c r="B22" s="35" t="n">
+        <v>46191</v>
+      </c>
+      <c r="C22" s="33" t="inlineStr">
+        <is>
+          <t>رسوم جوازات حسين مصطفى</t>
+        </is>
+      </c>
+      <c r="D22" s="34" t="n">
+        <v>163</v>
+      </c>
+      <c r="E22" s="33" t="inlineStr">
+        <is>
+          <t>إقامات ورسوم حكومية</t>
+        </is>
+      </c>
+      <c r="F22" s="33" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="33" t="n">
+        <v>8</v>
+      </c>
+      <c r="B23" s="35" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C23" s="33" t="inlineStr">
+        <is>
+          <t>إيجار مزرعة الرياض</t>
+        </is>
+      </c>
+      <c r="D23" s="34" t="n">
+        <v>150000</v>
+      </c>
+      <c r="E23" s="33" t="inlineStr">
+        <is>
+          <t>إيجار</t>
+        </is>
+      </c>
+      <c r="F23" s="33" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="33" t="n">
+        <v>9</v>
+      </c>
+      <c r="B24" s="35" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C24" s="33" t="inlineStr">
+        <is>
+          <t>رخص محمد عبدالمجيد</t>
+        </is>
+      </c>
+      <c r="D24" s="34" t="n">
+        <v>2425</v>
+      </c>
+      <c r="E24" s="33" t="inlineStr">
+        <is>
+          <t>إقامات ورسوم حكومية</t>
+        </is>
+      </c>
+      <c r="F24" s="33" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="33" t="n">
+        <v>10</v>
+      </c>
+      <c r="B25" s="35" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C25" s="33" t="inlineStr">
+        <is>
+          <t>رسوم جوازات</t>
+        </is>
+      </c>
+      <c r="D25" s="34" t="n">
+        <v>163</v>
+      </c>
+      <c r="E25" s="33" t="inlineStr">
+        <is>
+          <t>إقامات ورسوم حكومية</t>
+        </is>
+      </c>
+      <c r="F25" s="33" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="33" t="n">
+        <v>11</v>
+      </c>
+      <c r="B26" s="35" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C26" s="33" t="inlineStr">
+        <is>
+          <t>سداد مخالفات مرورية / عماد حمدي</t>
+        </is>
+      </c>
+      <c r="D26" s="34" t="n">
+        <v>863</v>
+      </c>
+      <c r="E26" s="33" t="inlineStr">
+        <is>
+          <t>مخالفات مرورية</t>
+        </is>
+      </c>
+      <c r="F26" s="33" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="B27" s="35" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C27" s="33" t="inlineStr">
+        <is>
+          <t>تجديد إقامة منير جمال</t>
+        </is>
+      </c>
+      <c r="D27" s="34" t="n">
+        <v>5175</v>
+      </c>
+      <c r="E27" s="33" t="inlineStr">
+        <is>
+          <t>إقامات ورسوم حكومية</t>
+        </is>
+      </c>
+      <c r="F27" s="33" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="33" t="n">
+        <v>13</v>
+      </c>
+      <c r="B28" s="35" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C28" s="33" t="inlineStr">
+        <is>
+          <t>رخص عمل عماد حمدي</t>
+        </is>
+      </c>
+      <c r="D28" s="34" t="n">
+        <v>2425</v>
+      </c>
+      <c r="E28" s="33" t="inlineStr">
+        <is>
+          <t>إقامات ورسوم حكومية</t>
+        </is>
+      </c>
+      <c r="F28" s="33" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="33" t="n">
+        <v>14</v>
+      </c>
+      <c r="B29" s="35" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C29" s="33" t="inlineStr">
+        <is>
+          <t>التأمين الطبي</t>
+        </is>
+      </c>
+      <c r="D29" s="34" t="n">
+        <v>258.87</v>
+      </c>
+      <c r="E29" s="33" t="inlineStr">
+        <is>
+          <t>تأمين طبي</t>
+        </is>
+      </c>
+      <c r="F29" s="33" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="33" t="n">
+        <v>15</v>
+      </c>
+      <c r="B30" s="35" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C30" s="33" t="inlineStr">
+        <is>
+          <t>شراء كفر للدينه 3010</t>
+        </is>
+      </c>
+      <c r="D30" s="34" t="n">
+        <v>400</v>
+      </c>
+      <c r="E30" s="33" t="inlineStr">
+        <is>
+          <t>مصاريف سيارات</t>
+        </is>
+      </c>
+      <c r="F30" s="33" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="33" t="n">
+        <v>16</v>
+      </c>
+      <c r="B31" s="35" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C31" s="33" t="inlineStr">
+        <is>
+          <t>سداد رخص العمل</t>
+        </is>
+      </c>
+      <c r="D31" s="34" t="n">
+        <v>2425</v>
+      </c>
+      <c r="E31" s="33" t="inlineStr">
+        <is>
+          <t>إقامات ورسوم حكومية</t>
+        </is>
+      </c>
+      <c r="F31" s="33" t="inlineStr">
+        <is>
+          <t>سداد رخص العمل بدون ذكر اسم العامل</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="33" t="n">
+        <v>17</v>
+      </c>
+      <c r="B32" s="35" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C32" s="33" t="inlineStr">
+        <is>
+          <t>رسوم جوازات محمد عبدالمجيد</t>
+        </is>
+      </c>
+      <c r="D32" s="34" t="n">
+        <v>163</v>
+      </c>
+      <c r="E32" s="33" t="inlineStr">
+        <is>
+          <t>إقامات ورسوم حكومية</t>
+        </is>
+      </c>
+      <c r="F32" s="33" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="B33" s="21" t="n">
+        <v>46235</v>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>رسوم الجوازات</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="n">
+        <v>163</v>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>إقامات ورسوم حكومية</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>⚠ بتاريخ 1-8-2026 بعد نهاية الفترة 31-7-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="inlineStr"/>
+      <c r="B34" s="15" t="inlineStr"/>
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>إجمالي المصاريف الإدارية 2026 (مطابق لتقرير العهدة 174,142.15)</t>
+        </is>
+      </c>
+      <c r="D34" s="16">
+        <f>SUM(D16:D33)</f>
+        <v/>
+      </c>
+      <c r="E34" s="15" t="n"/>
+      <c r="F34" s="15" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>منها خارج الفترة (بعد 31-7-2026)</t>
+        </is>
+      </c>
+      <c r="D35" s="36" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr"/>
+      <c r="B36" s="15" t="inlineStr"/>
+      <c r="C36" s="15" t="inlineStr">
+        <is>
+          <t>إجمالي 2026 حتى 31-7-2026</t>
+        </is>
+      </c>
+      <c r="D36" s="16">
+        <f>D34-D35</f>
+        <v/>
+      </c>
+      <c r="E36" s="15" t="n"/>
+      <c r="F36" s="15" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="31" t="inlineStr">
+        <is>
+          <t>ثالثاً: الديزل المدفوع من نسما الشرق لسيارات المناديب</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="32" t="inlineStr">
+        <is>
+          <t>السيارة</t>
+        </is>
+      </c>
+      <c r="B39" s="32" t="inlineStr">
+        <is>
+          <t>السائق</t>
+        </is>
+      </c>
+      <c r="C39" s="32" t="inlineStr">
+        <is>
+          <t>نوفمبر 2025</t>
+        </is>
+      </c>
+      <c r="D39" s="32" t="inlineStr">
+        <is>
+          <t>ديسمبر 2025</t>
+        </is>
+      </c>
+      <c r="E39" s="32" t="inlineStr">
+        <is>
+          <t>2026 حتى 31-7-2026</t>
+        </is>
+      </c>
+      <c r="F39" s="32" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="33" t="n">
+        <v>1219</v>
+      </c>
+      <c r="B40" s="33" t="inlineStr">
+        <is>
+          <t>عصمت الله خان</t>
+        </is>
+      </c>
+      <c r="C40" s="34" t="n">
+        <v>1840.94</v>
+      </c>
+      <c r="D40" s="34" t="n">
+        <v>1752.28</v>
+      </c>
+      <c r="E40" s="34" t="n">
+        <v>8017</v>
+      </c>
+      <c r="F40" s="34">
+        <f>C40+D40+E40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="33" t="n">
+        <v>3010</v>
+      </c>
+      <c r="B41" s="33" t="inlineStr">
+        <is>
+          <t>عماد حمدي</t>
+        </is>
+      </c>
+      <c r="C41" s="34" t="n">
+        <v>3464.26</v>
+      </c>
+      <c r="D41" s="34" t="n">
+        <v>3196.5</v>
+      </c>
+      <c r="E41" s="34" t="n">
+        <v>16871</v>
+      </c>
+      <c r="F41" s="34">
+        <f>C41+D41+E41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="inlineStr"/>
+      <c r="B42" s="15" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="C42" s="16">
+        <f>SUM(C40:C41)</f>
+        <v/>
+      </c>
+      <c r="D42" s="16">
+        <f>SUM(D40:D41)</f>
+        <v/>
+      </c>
+      <c r="E42" s="16">
+        <f>SUM(E40:E41)</f>
+        <v/>
+      </c>
+      <c r="F42" s="16">
+        <f>SUM(F40:F41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="31" t="inlineStr">
+        <is>
+          <t>الملخص</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="32" t="inlineStr"/>
+      <c r="B45" s="32" t="inlineStr"/>
+      <c r="C45" s="32" t="inlineStr">
+        <is>
+          <t>البند</t>
+        </is>
+      </c>
+      <c r="D45" s="32" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E45" s="32" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F45" s="32" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="33" t="inlineStr"/>
+      <c r="B46" s="33" t="inlineStr"/>
+      <c r="C46" s="33" t="inlineStr">
+        <is>
+          <t>المصاريف الإدارية</t>
+        </is>
+      </c>
+      <c r="D46" s="34">
+        <f>D12</f>
+        <v/>
+      </c>
+      <c r="E46" s="34">
+        <f>D36</f>
+        <v/>
+      </c>
+      <c r="F46" s="34">
+        <f>D46+E46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="33" t="inlineStr"/>
+      <c r="B47" s="33" t="inlineStr"/>
+      <c r="C47" s="33" t="inlineStr">
+        <is>
+          <t>الديزل</t>
+        </is>
+      </c>
+      <c r="D47" s="34">
+        <f>C42+D42</f>
+        <v/>
+      </c>
+      <c r="E47" s="34">
+        <f>E42</f>
+        <v/>
+      </c>
+      <c r="F47" s="34">
+        <f>D47+E47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr"/>
+      <c r="B48" s="15" t="inlineStr"/>
+      <c r="C48" s="15" t="inlineStr">
+        <is>
+          <t>الإجمالي المدفوع لمزرعة الرياض عن طريق تبوك</t>
+        </is>
+      </c>
+      <c r="D48" s="16">
+        <f>SUM(D46:D47)</f>
+        <v/>
+      </c>
+      <c r="E48" s="16">
+        <f>SUM(E46:E47)</f>
+        <v/>
+      </c>
+      <c r="F48" s="16">
+        <f>SUM(F46:F47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="29" t="inlineStr"/>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="29" t="inlineStr">
+        <is>
+          <t>ملاحظات:</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="29" t="inlineStr">
+        <is>
+          <t>1) إجمالي المصاريف الإدارية 2025 = 56,125.00 ومطابق للكشف. إجمالي 2026 = 174,142.15 ومطابق لتقرير العهدة، منها 163 بتاريخ 1-8-2026 خارج الفترة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="29" t="inlineStr">
+        <is>
+          <t>2) إيجار مزرعة الرياض 150,000 يمثل 86% من مصاريف 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="29" t="inlineStr">
+        <is>
+          <t>3) تقرير العهدة يوضح 18 صرفاً بدون أي تسوية معتمدة (Settled = 0) – الرصيد المتبقي بالعهدة 174,142.15، يعني لم تُقدم مستندات تسوية بعد.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="29" t="inlineStr">
+        <is>
+          <t>4) الديزل: إجمالي الشيت 35,141.98 وهو صحيح حسابياً. بيانات 2025 عن نوفمبر وديسمبر فقط، وبيانات 2026 إجمالي حتى 31-7-2026 بدون تفصيل شهري.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="29" t="inlineStr">
+        <is>
+          <t>5) مصاريف 2025 الإدارية بدون تواريخ تفصيلية في الكشف.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A52:F52"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="A55:F55"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2564,7 +3585,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7116,7 +8137,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add km transport cost receivable from Tabuk
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA2XXv3viuKc4AVC546mfn
</commit_message>
<xml_diff>
--- a/مراجعة_شيتات_المسحوبات_الرياض_تبوك.xlsx
+++ b/مراجعة_شيتات_المسحوبات_الرياض_تبوك.xlsx
@@ -21,9 +21,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -118,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -182,6 +181,10 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1429,7 +1432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1447,6 +1450,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="31" t="inlineStr">
         <is>
@@ -1673,6 +1677,7 @@
       <c r="E12" s="15" t="n"/>
       <c r="F12" s="15" t="n"/>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="31" t="inlineStr">
         <is>
@@ -2132,8 +2137,6 @@
       <c r="F34" s="15" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>منها خارج الفترة (بعد 31-7-2026)</t>
@@ -2158,6 +2161,7 @@
       <c r="E36" s="15" t="n"/>
       <c r="F36" s="15" t="n"/>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="31" t="inlineStr">
         <is>
@@ -2267,6 +2271,7 @@
         <v/>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" s="31" t="inlineStr">
         <is>
@@ -2406,20 +2411,124 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="31" t="inlineStr">
+        <is>
+          <t>رابعاً: تكاليف النقل خارج الرياض لصالح مزرعة تبوك (مديونية على مزرعة تبوك لصالح مزرعة الرياض)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="37" t="inlineStr"/>
+      <c r="B58" s="37" t="inlineStr"/>
+      <c r="C58" s="37" t="inlineStr">
+        <is>
+          <t>البيان</t>
+        </is>
+      </c>
+      <c r="D58" s="37" t="inlineStr">
+        <is>
+          <t>إجمالي الكيلومترات</t>
+        </is>
+      </c>
+      <c r="E58" s="37" t="inlineStr">
+        <is>
+          <t>تكلفة الكيلومتر</t>
+        </is>
+      </c>
+      <c r="F58" s="37" t="inlineStr">
+        <is>
+          <t>القيمة</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr"/>
+      <c r="B59" s="17" t="inlineStr"/>
+      <c r="C59" s="17" t="inlineStr">
+        <is>
+          <t>نقل خارج الرياض بسيارات مزرعة الرياض لصالح مزرعة تبوك</t>
+        </is>
+      </c>
+      <c r="D59" s="38" t="n">
+        <v>15290</v>
+      </c>
+      <c r="E59" s="19" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F59" s="19">
+        <f>D59*E59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="31" t="inlineStr">
+        <is>
+          <t>صافي الحساب بين المزرعتين (لهذه البنود)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="33" t="inlineStr"/>
+      <c r="B62" s="33" t="inlineStr"/>
+      <c r="C62" s="33" t="inlineStr">
+        <is>
+          <t>مصاريف إدارية وديزل دفعتها تبوك عن الرياض (مديونية على الرياض)</t>
+        </is>
+      </c>
+      <c r="D62" s="33" t="inlineStr"/>
+      <c r="E62" s="33" t="inlineStr"/>
+      <c r="F62" s="34">
+        <f>F48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="33" t="inlineStr"/>
+      <c r="B63" s="33" t="inlineStr"/>
+      <c r="C63" s="33" t="inlineStr">
+        <is>
+          <t>يُخصم: تكاليف النقل لصالح تبوك (مديونية على تبوك)</t>
+        </is>
+      </c>
+      <c r="D63" s="33" t="inlineStr"/>
+      <c r="E63" s="33" t="inlineStr"/>
+      <c r="F63" s="34">
+        <f>-F59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="15" t="inlineStr"/>
+      <c r="B64" s="15" t="inlineStr"/>
+      <c r="C64" s="15" t="inlineStr">
+        <is>
+          <t>الصافي المستحق لمزرعة تبوك على مزرعة الرياض</t>
+        </is>
+      </c>
+      <c r="D64" s="15" t="inlineStr"/>
+      <c r="E64" s="15" t="inlineStr"/>
+      <c r="F64" s="16">
+        <f>SUM(F62:F63)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="A54:F54"/>
     <mergeCell ref="A49:F49"/>
+    <mergeCell ref="A52:F52"/>
     <mergeCell ref="A51:F51"/>
-    <mergeCell ref="A52:F52"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A61:F61"/>
     <mergeCell ref="A50:F50"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A53:F53"/>
     <mergeCell ref="A55:F55"/>
+    <mergeCell ref="A57:F57"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove net balance section until all items are compiled
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA2XXv3viuKc4AVC546mfn
</commit_message>
<xml_diff>
--- a/مراجعة_شيتات_المسحوبات_الرياض_تبوك.xlsx
+++ b/مراجعة_شيتات_المسحوبات_الرياض_تبوك.xlsx
@@ -1432,7 +1432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2411,6 +2411,7 @@
         </is>
       </c>
     </row>
+    <row r="56"/>
     <row r="57">
       <c r="A57" s="31" t="inlineStr">
         <is>
@@ -2461,60 +2462,8 @@
         <v/>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="31" t="inlineStr">
-        <is>
-          <t>صافي الحساب بين المزرعتين (لهذه البنود)</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="33" t="inlineStr"/>
-      <c r="B62" s="33" t="inlineStr"/>
-      <c r="C62" s="33" t="inlineStr">
-        <is>
-          <t>مصاريف إدارية وديزل دفعتها تبوك عن الرياض (مديونية على الرياض)</t>
-        </is>
-      </c>
-      <c r="D62" s="33" t="inlineStr"/>
-      <c r="E62" s="33" t="inlineStr"/>
-      <c r="F62" s="34">
-        <f>F48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="33" t="inlineStr"/>
-      <c r="B63" s="33" t="inlineStr"/>
-      <c r="C63" s="33" t="inlineStr">
-        <is>
-          <t>يُخصم: تكاليف النقل لصالح تبوك (مديونية على تبوك)</t>
-        </is>
-      </c>
-      <c r="D63" s="33" t="inlineStr"/>
-      <c r="E63" s="33" t="inlineStr"/>
-      <c r="F63" s="34">
-        <f>-F59</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="15" t="inlineStr"/>
-      <c r="B64" s="15" t="inlineStr"/>
-      <c r="C64" s="15" t="inlineStr">
-        <is>
-          <t>الصافي المستحق لمزرعة تبوك على مزرعة الرياض</t>
-        </is>
-      </c>
-      <c r="D64" s="15" t="inlineStr"/>
-      <c r="E64" s="15" t="inlineStr"/>
-      <c r="F64" s="16">
-        <f>SUM(F62:F63)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="13">
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="A54:F54"/>
     <mergeCell ref="A49:F49"/>
@@ -2523,7 +2472,6 @@
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A61:F61"/>
     <mergeCell ref="A50:F50"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A53:F53"/>

</xml_diff>